<commit_message>
+ PLS-1.27-1, IDC-10F, BH-10R
</commit_message>
<xml_diff>
--- a/OurLib.xlsx
+++ b/OurLib.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\my-altium-library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B9CC371-FA56-4A75-8352-898E4875CCDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AD1F177-F807-424F-B788-8E7623505AD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="4215" windowWidth="21600" windowHeight="11385" tabRatio="500" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" tabRatio="500" firstSheet="8" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01 - Резисторы" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="252">
   <si>
     <t>Part Number</t>
   </si>
@@ -793,16 +793,36 @@
   </si>
   <si>
     <t>74HC165</t>
+  </si>
+  <si>
+    <t>IDC-10F</t>
+  </si>
+  <si>
+    <t>PLS-1.27-10</t>
+  </si>
+  <si>
+    <t>PLS-1.27-N10</t>
+  </si>
+  <si>
+    <t>PLS-1.27-F10</t>
+  </si>
+  <si>
+    <t>BH-10R</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <charset val="1"/>
     </font>
@@ -1687,7 +1707,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.85546875" style="1" customWidth="1"/>
@@ -2085,9 +2105,73 @@
         <v>168</v>
       </c>
     </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>